<commit_message>
Calibration edit to set MABAaSoF to 0.04
</commit_message>
<xml_diff>
--- a/InputData/elec/MABAaSoF/Max Annual Buildable Additions as Share of Fleet.xlsx
+++ b/InputData/elec/MABAaSoF/Max Annual Buildable Additions as Share of Fleet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-analysis\InputData\elec\MABAaSoF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\MABAaSoF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E05C5D-90AB-480E-943F-31A7C9FECFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC218B0-6624-4E4D-ACFA-8C30D2490331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="26640" windowHeight="15615" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -490,7 +490,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Calibration edit to set MABAaSoF to 0.04"
This reverts commit d606c21743235fe38500ff44bb1534cfe99fd145.
</commit_message>
<xml_diff>
--- a/InputData/elec/MABAaSoF/Max Annual Buildable Additions as Share of Fleet.xlsx
+++ b/InputData/elec/MABAaSoF/Max Annual Buildable Additions as Share of Fleet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\MABAaSoF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-analysis\InputData\elec\MABAaSoF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC218B0-6624-4E4D-ACFA-8C30D2490331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E05C5D-90AB-480E-943F-31A7C9FECFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="26640" windowHeight="15615" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -490,7 +490,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>